<commit_message>
Pipeline map: Products SE Pipeline name; draw press-reported capacities
Plantation is labelled by its current name, the Products SE Pipeline
(Kinder Morgan 10-K for 2025). Olympic, Laurel, CALNEV, Centennial and
Mid-Valley are drawn at their reported capacity; the spreadsheet keeps
each figure's source type.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E3iewxRZcp5cfzqxTzR3MF
</commit_message>
<xml_diff>
--- a/data/pipelines/pipeline_capacity_sources.xlsx
+++ b/data/pipelines/pipeline_capacity_sources.xlsx
@@ -537,14 +537,14 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Source type: Official (EIA), Company SEC filing (10-K), Company website, Derived, Industry reference, or Press. Press figures could not be confirmed from an operator or official document, so those lines are drawn thin. The one Industry reference (Colonial north of Greensboro, NC) is drawn, because EIA publishes no figure for that stretch and a thin line would show Colonial ending in North Carolina.</t>
+          <t>Source type: Official (EIA), Company SEC filing (10-K), Company website, Derived, Industry reference, or Press. Press and industry-reference figures could not be confirmed from an operator or official document; they are the best figures available and are drawn at the reported value.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Width on map: 'No (thin)' lines appear on the map at a fixed thin width.</t>
+          <t>Width on map: 'No (thin)' lines have no capacity figure from any source and appear at a fixed thin width.</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Plantation Pipe Line</t>
+          <t>Products SE Pipeline (formerly Plantation)</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
-          <t>Now called the Products (SE) Pipeline. Earlier: about 710,000 b/d after a 2001 expansion (Kinder Morgan Energy Partners 10-K405 for 2001: https://www.sec.gov/Archives/edgar/data/888228/000095012902000816/h94309e10-k405.txt). Drawn on the mainline only; laterals are thin</t>
+          <t>Renamed from Plantation: Kinder Morgan's 10-K for 2025 lists the "Products (SE) pipeline" (3,181 miles, 51% owned via Products (SE) Pipe Line Corporation): https://www.sec.gov/Archives/edgar/data/1506307/000150630726000011/kmi-20251231.htm. Earlier: about 710,000 b/d after a 2001 expansion (Kinder Morgan Energy Partners 10-K405 for 2001: https://www.sec.gov/Archives/edgar/data/888228/000095012902000816/h94309e10-k405.txt). Drawn on the mainline only; laterals are thin</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
@@ -1482,12 +1482,12 @@
       <c r="J14" s="6" t="inlineStr"/>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>Not confirmed from an operator or official document; drawn thin</t>
+          <t>Not confirmed from an operator or official document; drawn at the reported figure</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>No (thin)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="M14" s="6" t="n">
@@ -1537,12 +1537,12 @@
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Not confirmed from an operator or official document; drawn thin</t>
+          <t>Not confirmed from an operator or official document; drawn at the reported figure</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>No (thin)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="M15" s="2" t="n">
@@ -1592,12 +1592,12 @@
       <c r="J16" s="6" t="inlineStr"/>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>Not confirmed from an operator or official document; drawn thin</t>
+          <t>Not confirmed from an operator or official document; drawn at the reported figure</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
-          <t>No (thin)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="M16" s="6" t="n">
@@ -1651,12 +1651,12 @@
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Current operating status not confirmed; drawn thin</t>
+          <t>Current operating status not confirmed; drawn at its 2002 design capacity</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>No (thin)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="M17" s="2" t="n">
@@ -3490,12 +3490,12 @@
       <c r="J48" s="6" t="inlineStr"/>
       <c r="K48" s="6" t="inlineStr">
         <is>
-          <t>Not confirmed from an operator or official document; drawn thin</t>
+          <t>Not confirmed from an operator or official document; drawn at the reported figure</t>
         </is>
       </c>
       <c r="L48" s="6" t="inlineStr">
         <is>
-          <t>No (thin)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="M48" s="6" t="n">

</xml_diff>

<commit_message>
Pipeline map: Products SE Pipeline name; draw press-reported capacities (#21)
Plantation is labelled by its current name, the Products SE Pipeline
(Kinder Morgan 10-K for 2025). Olympic, Laurel, CALNEV, Centennial and
Mid-Valley are drawn at their reported capacity; the spreadsheet keeps
each figure's source type.


Claude-Session: https://claude.ai/code/session_01E3iewxRZcp5cfzqxTzR3MF

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/pipelines/pipeline_capacity_sources.xlsx
+++ b/data/pipelines/pipeline_capacity_sources.xlsx
@@ -537,14 +537,14 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Source type: Official (EIA), Company SEC filing (10-K), Company website, Derived, Industry reference, or Press. Press figures could not be confirmed from an operator or official document, so those lines are drawn thin. The one Industry reference (Colonial north of Greensboro, NC) is drawn, because EIA publishes no figure for that stretch and a thin line would show Colonial ending in North Carolina.</t>
+          <t>Source type: Official (EIA), Company SEC filing (10-K), Company website, Derived, Industry reference, or Press. Press and industry-reference figures could not be confirmed from an operator or official document; they are the best figures available and are drawn at the reported value.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Width on map: 'No (thin)' lines appear on the map at a fixed thin width.</t>
+          <t>Width on map: 'No (thin)' lines have no capacity figure from any source and appear at a fixed thin width.</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Plantation Pipe Line</t>
+          <t>Products SE Pipeline (formerly Plantation)</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
-          <t>Now called the Products (SE) Pipeline. Earlier: about 710,000 b/d after a 2001 expansion (Kinder Morgan Energy Partners 10-K405 for 2001: https://www.sec.gov/Archives/edgar/data/888228/000095012902000816/h94309e10-k405.txt). Drawn on the mainline only; laterals are thin</t>
+          <t>Renamed from Plantation: Kinder Morgan's 10-K for 2025 lists the "Products (SE) pipeline" (3,181 miles, 51% owned via Products (SE) Pipe Line Corporation): https://www.sec.gov/Archives/edgar/data/1506307/000150630726000011/kmi-20251231.htm. Earlier: about 710,000 b/d after a 2001 expansion (Kinder Morgan Energy Partners 10-K405 for 2001: https://www.sec.gov/Archives/edgar/data/888228/000095012902000816/h94309e10-k405.txt). Drawn on the mainline only; laterals are thin</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
@@ -1482,12 +1482,12 @@
       <c r="J14" s="6" t="inlineStr"/>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>Not confirmed from an operator or official document; drawn thin</t>
+          <t>Not confirmed from an operator or official document; drawn at the reported figure</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>No (thin)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="M14" s="6" t="n">
@@ -1537,12 +1537,12 @@
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Not confirmed from an operator or official document; drawn thin</t>
+          <t>Not confirmed from an operator or official document; drawn at the reported figure</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>No (thin)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="M15" s="2" t="n">
@@ -1592,12 +1592,12 @@
       <c r="J16" s="6" t="inlineStr"/>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>Not confirmed from an operator or official document; drawn thin</t>
+          <t>Not confirmed from an operator or official document; drawn at the reported figure</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
-          <t>No (thin)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="M16" s="6" t="n">
@@ -1651,12 +1651,12 @@
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Current operating status not confirmed; drawn thin</t>
+          <t>Current operating status not confirmed; drawn at its 2002 design capacity</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>No (thin)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="M17" s="2" t="n">
@@ -3490,12 +3490,12 @@
       <c r="J48" s="6" t="inlineStr"/>
       <c r="K48" s="6" t="inlineStr">
         <is>
-          <t>Not confirmed from an operator or official document; drawn thin</t>
+          <t>Not confirmed from an operator or official document; drawn at the reported figure</t>
         </is>
       </c>
       <c r="L48" s="6" t="inlineStr">
         <is>
-          <t>No (thin)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="M48" s="6" t="n">

</xml_diff>

<commit_message>
Pipeline map: routes reach their cities; more capacities; city labels
EIA's routes are simplified sketches, so some Western lines stopped short
of the city they supply (Olympic 14 miles from Seattle, CALNEV 8 from Las
Vegas). Each refined-product route's nearest point to a Western terminal
city within 20 miles now snaps onto it, and 13 cities are labelled.

Adds 16 capacity rows (Trans Mountain 890,000 b/d per the Canada Energy
Regulator; Keystone's legs to Patoka and Cushing; Zydeco, Permian Express
2, Marathon's crude lines from Patoka, Red River; Phillips 66 crude lines
and Seminoe; Colonial to Nashville; three NuStar lines) and corrects
Basin to its Colorado City to Cushing capacity. Trans Mountain is drawn
once, as crude. Other maps render pixel-identical.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E3iewxRZcp5cfzqxTzR3MF
</commit_message>
<xml_diff>
--- a/data/pipelines/pipeline_capacity_sources.xlsx
+++ b/data/pipelines/pipeline_capacity_sources.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Pipelines" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pipelines'!$A$1:$M$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pipelines'!$A$1:$M$112</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="B13" s="4">
-        <f>COUNTA(Pipelines!B2:B96)</f>
+        <f>COUNTA(Pipelines!B2:B112)</f>
         <v/>
       </c>
     </row>
@@ -576,7 +576,7 @@
         </is>
       </c>
       <c r="B14" s="4">
-        <f>COUNTIF(Pipelines!L2:L96,"Yes")</f>
+        <f>COUNTIF(Pipelines!L2:L112,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="B15" s="4">
-        <f>SUMIFS(Pipelines!D2:D96,Pipelines!A2:A96,"Refined products",Pipelines!L2:L96,"Yes")</f>
+        <f>SUMIFS(Pipelines!D2:D112,Pipelines!A2:A112,"Refined products",Pipelines!L2:L112,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="B16" s="4">
-        <f>SUMIFS(Pipelines!D2:D96,Pipelines!A2:A96,"Crude oil",Pipelines!L2:L96,"Yes")</f>
+        <f>SUMIFS(Pipelines!D2:D112,Pipelines!A2:A112,"Crude oil",Pipelines!L2:L112,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -630,7 +630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M96"/>
+  <dimension ref="A1:M112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3315,16 +3315,16 @@
         </is>
       </c>
       <c r="D45" s="9" t="n">
-        <v>600000</v>
+        <v>450000</v>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Capacity (Wink to Midland segment)</t>
+          <t>Capacity (Colorado City to Cushing segment)</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>EIA, Liquids pipeline projects database (ID 90)</t>
+          <t>EIA, Liquids pipeline projects database (IDs 19 and 90)</t>
         </is>
       </c>
       <c r="I45" s="10" t="inlineStr">
@@ -3344,12 +3344,12 @@
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>bring total capacity from 240,000 b/d to 600,000 b/d</t>
+          <t>Segment from Colorado City, Texas, to Cushing, Oklahoma, had its capacity increased from 400,000 b/d to 450,000 b/d.</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>This figure is for the Wink to Midland segment; the segment north to Cushing is smaller</t>
+          <t>EIA draws Basin as one route from the Permian to Cushing; the Wink to Midland segment was expanded to 600,000 b/d in 2015 (ID 90)</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr">
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="M45" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -6430,8 +6430,988 @@
         <v>1</v>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>Refined products</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>Colonial Lines 19 and 20 (Atlanta to Nashville)</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Atlanta, GA via Chattanooga to Nashville, TN</t>
+        </is>
+      </c>
+      <c r="D97" s="9" t="n">
+        <v>250000</v>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>Throughput (2015, EIA range 250,000 to 300,000)</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>Official (EIA study)</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>EIA, PADDs 2 and 4 Transportation Fuels Markets, Jan 2017, Table 18</t>
+        </is>
+      </c>
+      <c r="I97" s="10" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/analysis/transportationfuels/padd2n4/pdf/transportation_fuels.pdf</t>
+        </is>
+      </c>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>Colonial Pipeline Line 19 Atlanta, GA Chattanooga Jct./Nashville, TN 10/12 250,000 - 300,000</t>
+        </is>
+      </c>
+      <c r="K97" s="2" t="inlineStr">
+        <is>
+          <t>Drawn at the low end of EIA's range</t>
+        </is>
+      </c>
+      <c r="L97" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M97" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="6" t="inlineStr">
+        <is>
+          <t>Refined products</t>
+        </is>
+      </c>
+      <c r="B98" s="6" t="inlineStr">
+        <is>
+          <t>Seminoe Pipeline</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="inlineStr">
+        <is>
+          <t>Billings, MT to Casper and Sinclair, WY</t>
+        </is>
+      </c>
+      <c r="D98" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="E98" s="6" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F98" s="6" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G98" s="6" t="inlineStr">
+        <is>
+          <t>Company SEC filing</t>
+        </is>
+      </c>
+      <c r="H98" s="6" t="inlineStr">
+        <is>
+          <t>Phillips 66, Form 10-K for 2025, pipeline table</t>
+        </is>
+      </c>
+      <c r="I98" s="8" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1534701/000153470126000006/psx-20251231.htm</t>
+        </is>
+      </c>
+      <c r="J98" s="6" t="inlineStr">
+        <is>
+          <t>Seminoe Montana/Wyoming 100 342 50</t>
+        </is>
+      </c>
+      <c r="K98" s="6" t="inlineStr">
+        <is>
+          <t>The EIA route layer spells it "Seminole"</t>
+        </is>
+      </c>
+      <c r="L98" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M98" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>Refined products</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>NuStar, McKee to Southlake (Dallas–Fort Worth)</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>McKee refinery (Sunray, TX) to Southlake, TX</t>
+        </is>
+      </c>
+      <c r="D99" s="9" t="n">
+        <v>26000</v>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>Official (EIA study)</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>EIA, East Coast and Gulf Coast Transportation Fuels Markets (prepared by ICF), Feb 2016, Table 30</t>
+        </is>
+      </c>
+      <c r="I99" s="10" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/analysis/transportationfuels/padd1n3/pdf/transportation_fuels_padd1n3.pdf</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>McKee, TX Southlake, TX 375 26,000</t>
+        </is>
+      </c>
+      <c r="K99" s="2" t="inlineStr"/>
+      <c r="L99" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M99" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="6" t="inlineStr">
+        <is>
+          <t>Refined products</t>
+        </is>
+      </c>
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>NuStar, McKee to El Paso</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="inlineStr">
+        <is>
+          <t>McKee refinery (Sunray, TX) to El Paso, TX</t>
+        </is>
+      </c>
+      <c r="D100" s="7" t="n">
+        <v>42000</v>
+      </c>
+      <c r="E100" s="6" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F100" s="6" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="G100" s="6" t="inlineStr">
+        <is>
+          <t>Official (EIA study)</t>
+        </is>
+      </c>
+      <c r="H100" s="6" t="inlineStr">
+        <is>
+          <t>EIA, East Coast and Gulf Coast Transportation Fuels Markets (prepared by ICF), Feb 2016, Table 30</t>
+        </is>
+      </c>
+      <c r="I100" s="8" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/analysis/transportationfuels/padd1n3/pdf/transportation_fuels_padd1n3.pdf</t>
+        </is>
+      </c>
+      <c r="J100" s="6" t="inlineStr">
+        <is>
+          <t>McKee, TX El Paso, TX 408 42,000</t>
+        </is>
+      </c>
+      <c r="K100" s="6" t="inlineStr"/>
+      <c r="L100" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M100" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>Refined products</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>NuStar, Three Rivers to San Antonio</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>Three Rivers, TX to San Antonio, TX</t>
+        </is>
+      </c>
+      <c r="D101" s="9" t="n">
+        <v>33500</v>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>Official (EIA study)</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>EIA, East Coast and Gulf Coast Transportation Fuels Markets (prepared by ICF), Feb 2016, Table 26</t>
+        </is>
+      </c>
+      <c r="I101" s="10" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/analysis/transportationfuels/padd1n3/pdf/transportation_fuels_padd1n3.pdf</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>Three Rivers, TX San Antonio, TX 85 33,500</t>
+        </is>
+      </c>
+      <c r="K101" s="2" t="inlineStr"/>
+      <c r="L101" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M101" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="6" t="inlineStr">
+        <is>
+          <t>Crude oil</t>
+        </is>
+      </c>
+      <c r="B102" s="6" t="inlineStr">
+        <is>
+          <t>Keystone Pipeline, Steele City to Patoka</t>
+        </is>
+      </c>
+      <c r="C102" s="6" t="inlineStr">
+        <is>
+          <t>Steele City, NE to Patoka, IL</t>
+        </is>
+      </c>
+      <c r="D102" s="7" t="n">
+        <v>435000</v>
+      </c>
+      <c r="E102" s="6" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F102" s="6" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="G102" s="6" t="inlineStr">
+        <is>
+          <t>Official (EIA)</t>
+        </is>
+      </c>
+      <c r="H102" s="6" t="inlineStr">
+        <is>
+          <t>EIA, Liquids pipeline projects database (ID 2)</t>
+        </is>
+      </c>
+      <c r="I102" s="8" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/petroleum/xls/EIA_LiqPipProject.xlsx</t>
+        </is>
+      </c>
+      <c r="J102" s="6" t="inlineStr">
+        <is>
+          <t>Goes from Hardisty in Alberta, Canada, down through Steele City, Nebraska, and to Patoka, Illinois. [Added capacity 435,000 b/d]</t>
+        </is>
+      </c>
+      <c r="K102" s="6" t="inlineStr"/>
+      <c r="L102" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M102" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>Crude oil</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>Keystone Pipeline, Steele City to Cushing</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>Steele City, NE to Cushing, OK</t>
+        </is>
+      </c>
+      <c r="D103" s="9" t="n">
+        <v>156000</v>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>Official (EIA)</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>EIA, Liquids pipeline projects database (ID 3)</t>
+        </is>
+      </c>
+      <c r="I103" s="10" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/petroleum/xls/EIA_LiqPipProject.xlsx</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t>Extended existing pipeline from Steele City, Nebraska, to Cushing, Oklahoma, and brought capacity of the entire system up to 591,000 b/d. [Added capacity 156,000 b/d]</t>
+        </is>
+      </c>
+      <c r="K103" s="2" t="inlineStr"/>
+      <c r="L103" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M103" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="6" t="inlineStr">
+        <is>
+          <t>Crude oil</t>
+        </is>
+      </c>
+      <c r="B104" s="6" t="inlineStr">
+        <is>
+          <t>Zydeco Pipeline (Houston to Houma)</t>
+        </is>
+      </c>
+      <c r="C104" s="6" t="inlineStr">
+        <is>
+          <t>Houston, TX via Port Neches, TX to Houma, LA</t>
+        </is>
+      </c>
+      <c r="D104" s="7" t="n">
+        <v>375000</v>
+      </c>
+      <c r="E104" s="6" t="inlineStr">
+        <is>
+          <t>Capacity (Port Neches to Houma segment)</t>
+        </is>
+      </c>
+      <c r="F104" s="6" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="G104" s="6" t="inlineStr">
+        <is>
+          <t>Official (EIA)</t>
+        </is>
+      </c>
+      <c r="H104" s="6" t="inlineStr">
+        <is>
+          <t>EIA, Liquids pipeline projects database (IDs 36 and 114)</t>
+        </is>
+      </c>
+      <c r="I104" s="8" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/petroleum/xls/EIA_LiqPipProject.xlsx</t>
+        </is>
+      </c>
+      <c r="J104" s="6" t="inlineStr">
+        <is>
+          <t>Increased capacity of Port Neches, Texas, to Houma, Louisiana, segment from 360,000 b/d to 375,000 b/d.</t>
+        </is>
+      </c>
+      <c r="K104" s="6" t="inlineStr">
+        <is>
+          <t>Houston to Port Neches segment: 250,000 b/d (ID 36)</t>
+        </is>
+      </c>
+      <c r="L104" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M104" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>Crude oil</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Permian Express 2</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>Colorado City, TX to Corsicana, TX</t>
+        </is>
+      </c>
+      <c r="D105" s="9" t="n">
+        <v>230000</v>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>Official (EIA)</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>EIA, Liquids pipeline projects database (ID 84)</t>
+        </is>
+      </c>
+      <c r="I105" s="10" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/petroleum/xls/EIA_LiqPipProject.xlsx</t>
+        </is>
+      </c>
+      <c r="J105" s="2" t="inlineStr">
+        <is>
+          <t>Garden City, Texas, to Colorado City, Texas, segment has 20-inch diameter pipeline, Colorado City to Corsicana, Texas, has 24-inch diameter pipeline. [Added capacity 230,000 b/d]</t>
+        </is>
+      </c>
+      <c r="K105" s="2" t="inlineStr"/>
+      <c r="L105" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M105" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="6" t="inlineStr">
+        <is>
+          <t>Crude oil</t>
+        </is>
+      </c>
+      <c r="B106" s="6" t="inlineStr">
+        <is>
+          <t>Marathon, Patoka to Catlettsburg</t>
+        </is>
+      </c>
+      <c r="C106" s="6" t="inlineStr">
+        <is>
+          <t>Patoka, IL via Owensboro, KY to Catlettsburg, KY</t>
+        </is>
+      </c>
+      <c r="D106" s="7" t="n">
+        <v>270000</v>
+      </c>
+      <c r="E106" s="6" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F106" s="6" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="G106" s="6" t="inlineStr">
+        <is>
+          <t>Official (EIA)</t>
+        </is>
+      </c>
+      <c r="H106" s="6" t="inlineStr">
+        <is>
+          <t>EIA, Liquids pipeline projects database (ID 22)</t>
+        </is>
+      </c>
+      <c r="I106" s="8" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/petroleum/xls/EIA_LiqPipProject.xlsx</t>
+        </is>
+      </c>
+      <c r="J106" s="6" t="inlineStr">
+        <is>
+          <t>Capacity increased from 256,000 b/d to 270,000 b/d.</t>
+        </is>
+      </c>
+      <c r="K106" s="6" t="inlineStr"/>
+      <c r="L106" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M106" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>Crude oil</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>Marathon, Patoka to Lima and Canton</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>Patoka, IL to Lima and Canton, OH</t>
+        </is>
+      </c>
+      <c r="D107" s="9" t="n">
+        <v>267000</v>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>Capacity (Patoka to Lima)</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>Official (EIA)</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>EIA, Liquids pipeline projects database (ID 111)</t>
+        </is>
+      </c>
+      <c r="I107" s="10" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/petroleum/xls/EIA_LiqPipProject.xlsx</t>
+        </is>
+      </c>
+      <c r="J107" s="2" t="inlineStr">
+        <is>
+          <t>Capacity increased from 249,000 b/d to 267,000 b/d.</t>
+        </is>
+      </c>
+      <c r="K107" s="2" t="inlineStr">
+        <is>
+          <t>EIA route continues past Lima to Canton</t>
+        </is>
+      </c>
+      <c r="L107" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M107" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="6" t="inlineStr">
+        <is>
+          <t>Crude oil</t>
+        </is>
+      </c>
+      <c r="B108" s="6" t="inlineStr">
+        <is>
+          <t>Red River Pipeline</t>
+        </is>
+      </c>
+      <c r="C108" s="6" t="inlineStr">
+        <is>
+          <t>Cushing, OK to Longview, TX</t>
+        </is>
+      </c>
+      <c r="D108" s="7" t="n">
+        <v>235000</v>
+      </c>
+      <c r="E108" s="6" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F108" s="6" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G108" s="6" t="inlineStr">
+        <is>
+          <t>Company SEC filing</t>
+        </is>
+      </c>
+      <c r="H108" s="6" t="inlineStr">
+        <is>
+          <t>Plains All American, Form 10-K for 2025</t>
+        </is>
+      </c>
+      <c r="I108" s="8" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1070423/000107042326000014/paa-20251231.htm</t>
+        </is>
+      </c>
+      <c r="J108" s="6" t="inlineStr">
+        <is>
+          <t>The Red River Pipeline is an approximately 235,000 barrel per day capacity pipeline that extends from our Cushing Terminal in Oklahoma to Longview, Texas</t>
+        </is>
+      </c>
+      <c r="K108" s="6" t="inlineStr">
+        <is>
+          <t>EIA route layer label: "CK Red River"</t>
+        </is>
+      </c>
+      <c r="L108" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M108" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>Crude oil</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>Phillips 66 Oklahoma Crude system</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>Wichita Falls, TX to Ponca City, OK</t>
+        </is>
+      </c>
+      <c r="D109" s="9" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>Company SEC filing</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>Phillips 66, Form 10-K for 2025, pipeline table</t>
+        </is>
+      </c>
+      <c r="I109" s="10" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1534701/000153470126000006/psx-20251231.htm</t>
+        </is>
+      </c>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
+          <t>Oklahoma Crude Texas/Oklahoma 100 217 100</t>
+        </is>
+      </c>
+      <c r="K109" s="2" t="inlineStr">
+        <is>
+          <t>Matched to the EIA route by operator and endpoints</t>
+        </is>
+      </c>
+      <c r="L109" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M109" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="6" t="inlineStr">
+        <is>
+          <t>Crude oil</t>
+        </is>
+      </c>
+      <c r="B110" s="6" t="inlineStr">
+        <is>
+          <t>Phillips 66 West Texas Crude system</t>
+        </is>
+      </c>
+      <c r="C110" s="6" t="inlineStr">
+        <is>
+          <t>Odessa, TX to Borger, TX</t>
+        </is>
+      </c>
+      <c r="D110" s="7" t="n">
+        <v>140000</v>
+      </c>
+      <c r="E110" s="6" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F110" s="6" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G110" s="6" t="inlineStr">
+        <is>
+          <t>Company SEC filing</t>
+        </is>
+      </c>
+      <c r="H110" s="6" t="inlineStr">
+        <is>
+          <t>Phillips 66, Form 10-K for 2025, pipeline table</t>
+        </is>
+      </c>
+      <c r="I110" s="8" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1534701/000153470126000006/psx-20251231.htm</t>
+        </is>
+      </c>
+      <c r="J110" s="6" t="inlineStr">
+        <is>
+          <t>West Texas Crude Texas 100 1,079 140</t>
+        </is>
+      </c>
+      <c r="K110" s="6" t="inlineStr">
+        <is>
+          <t>Matched to the EIA route by operator and endpoints</t>
+        </is>
+      </c>
+      <c r="L110" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M110" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>Crude oil</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>Phillips 66 California Line 200</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>San Joaquin Valley to Rodeo (San Francisco Bay), CA</t>
+        </is>
+      </c>
+      <c r="D111" s="9" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>Company SEC filing</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>Phillips 66, Form 10-K for 2025, pipeline table</t>
+        </is>
+      </c>
+      <c r="I111" s="10" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1534701/000153470126000006/psx-20251231.htm</t>
+        </is>
+      </c>
+      <c r="J111" s="2" t="inlineStr">
+        <is>
+          <t>Line 200 California 100 228 100</t>
+        </is>
+      </c>
+      <c r="K111" s="2" t="inlineStr">
+        <is>
+          <t>Matched to the EIA route by operator and endpoints</t>
+        </is>
+      </c>
+      <c r="L111" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M111" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="6" t="inlineStr">
+        <is>
+          <t>Crude oil</t>
+        </is>
+      </c>
+      <c r="B112" s="6" t="inlineStr">
+        <is>
+          <t>Trans Mountain Pipeline</t>
+        </is>
+      </c>
+      <c r="C112" s="6" t="inlineStr">
+        <is>
+          <t>Edmonton, AB to Burnaby (Vancouver), BC</t>
+        </is>
+      </c>
+      <c r="D112" s="7" t="n">
+        <v>890000</v>
+      </c>
+      <c r="E112" s="6" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F112" s="6" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="G112" s="6" t="inlineStr">
+        <is>
+          <t>Official (Canada Energy Regulator)</t>
+        </is>
+      </c>
+      <c r="H112" s="6" t="inlineStr">
+        <is>
+          <t>Canada Energy Regulator, Market Snapshot (2025): Trans Mountain Expansion eases pipeline constraints</t>
+        </is>
+      </c>
+      <c r="I112" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cer-rec.gc.ca/en/data-analysis/energy-markets/market-snapshots/2025/market-snapshot-trans-mountain-expansion-eases-pipeline-constraints-and-increases-exports-to-overseas-markets.html</t>
+        </is>
+      </c>
+      <c r="J112" s="6" t="inlineStr">
+        <is>
+          <t>The Trans Mountain Expansion Project came online in May 2024, nearly tripling the capacity of the Trans Mountain System to a total of 890 thousand barrels per day.</t>
+        </is>
+      </c>
+      <c r="K112" s="6" t="inlineStr">
+        <is>
+          <t>Now owned by Trans Mountain Corporation (Canadian government); the EIA layer still lists Kinder Morgan. Also listed in EIA's product layer, where it is left off to avoid drawing it twice</t>
+        </is>
+      </c>
+      <c r="L112" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M112" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M96"/>
+  <autoFilter ref="A1:M112"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId2"/>
@@ -6528,6 +7508,22 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I94" r:id="rId93"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I95" r:id="rId94"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I104" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I107" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I108" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I112" r:id="rId111"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Pipeline map: routes reach their cities; more capacities; city labels (#23)
EIA's routes are simplified sketches, so some Western lines stopped short
of the city they supply (Olympic 14 miles from Seattle, CALNEV 8 from Las
Vegas). Each refined-product route's nearest point to a Western terminal
city within 20 miles now snaps onto it, and 13 cities are labelled.

Adds 16 capacity rows (Trans Mountain 890,000 b/d per the Canada Energy
Regulator; Keystone's legs to Patoka and Cushing; Zydeco, Permian Express
2, Marathon's crude lines from Patoka, Red River; Phillips 66 crude lines
and Seminoe; Colonial to Nashville; three NuStar lines) and corrects
Basin to its Colorado City to Cushing capacity. Trans Mountain is drawn
once, as crude. Other maps render pixel-identical.


Claude-Session: https://claude.ai/code/session_01E3iewxRZcp5cfzqxTzR3MF

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/pipelines/pipeline_capacity_sources.xlsx
+++ b/data/pipelines/pipeline_capacity_sources.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Pipelines" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pipelines'!$A$1:$M$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pipelines'!$A$1:$M$112</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="B13" s="4">
-        <f>COUNTA(Pipelines!B2:B96)</f>
+        <f>COUNTA(Pipelines!B2:B112)</f>
         <v/>
       </c>
     </row>
@@ -576,7 +576,7 @@
         </is>
       </c>
       <c r="B14" s="4">
-        <f>COUNTIF(Pipelines!L2:L96,"Yes")</f>
+        <f>COUNTIF(Pipelines!L2:L112,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="B15" s="4">
-        <f>SUMIFS(Pipelines!D2:D96,Pipelines!A2:A96,"Refined products",Pipelines!L2:L96,"Yes")</f>
+        <f>SUMIFS(Pipelines!D2:D112,Pipelines!A2:A112,"Refined products",Pipelines!L2:L112,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="B16" s="4">
-        <f>SUMIFS(Pipelines!D2:D96,Pipelines!A2:A96,"Crude oil",Pipelines!L2:L96,"Yes")</f>
+        <f>SUMIFS(Pipelines!D2:D112,Pipelines!A2:A112,"Crude oil",Pipelines!L2:L112,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -630,7 +630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M96"/>
+  <dimension ref="A1:M112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3315,16 +3315,16 @@
         </is>
       </c>
       <c r="D45" s="9" t="n">
-        <v>600000</v>
+        <v>450000</v>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Capacity (Wink to Midland segment)</t>
+          <t>Capacity (Colorado City to Cushing segment)</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>EIA, Liquids pipeline projects database (ID 90)</t>
+          <t>EIA, Liquids pipeline projects database (IDs 19 and 90)</t>
         </is>
       </c>
       <c r="I45" s="10" t="inlineStr">
@@ -3344,12 +3344,12 @@
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>bring total capacity from 240,000 b/d to 600,000 b/d</t>
+          <t>Segment from Colorado City, Texas, to Cushing, Oklahoma, had its capacity increased from 400,000 b/d to 450,000 b/d.</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>This figure is for the Wink to Midland segment; the segment north to Cushing is smaller</t>
+          <t>EIA draws Basin as one route from the Permian to Cushing; the Wink to Midland segment was expanded to 600,000 b/d in 2015 (ID 90)</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr">
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="M45" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -6430,8 +6430,988 @@
         <v>1</v>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>Refined products</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>Colonial Lines 19 and 20 (Atlanta to Nashville)</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Atlanta, GA via Chattanooga to Nashville, TN</t>
+        </is>
+      </c>
+      <c r="D97" s="9" t="n">
+        <v>250000</v>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>Throughput (2015, EIA range 250,000 to 300,000)</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>Official (EIA study)</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>EIA, PADDs 2 and 4 Transportation Fuels Markets, Jan 2017, Table 18</t>
+        </is>
+      </c>
+      <c r="I97" s="10" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/analysis/transportationfuels/padd2n4/pdf/transportation_fuels.pdf</t>
+        </is>
+      </c>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>Colonial Pipeline Line 19 Atlanta, GA Chattanooga Jct./Nashville, TN 10/12 250,000 - 300,000</t>
+        </is>
+      </c>
+      <c r="K97" s="2" t="inlineStr">
+        <is>
+          <t>Drawn at the low end of EIA's range</t>
+        </is>
+      </c>
+      <c r="L97" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M97" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="6" t="inlineStr">
+        <is>
+          <t>Refined products</t>
+        </is>
+      </c>
+      <c r="B98" s="6" t="inlineStr">
+        <is>
+          <t>Seminoe Pipeline</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="inlineStr">
+        <is>
+          <t>Billings, MT to Casper and Sinclair, WY</t>
+        </is>
+      </c>
+      <c r="D98" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="E98" s="6" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F98" s="6" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G98" s="6" t="inlineStr">
+        <is>
+          <t>Company SEC filing</t>
+        </is>
+      </c>
+      <c r="H98" s="6" t="inlineStr">
+        <is>
+          <t>Phillips 66, Form 10-K for 2025, pipeline table</t>
+        </is>
+      </c>
+      <c r="I98" s="8" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1534701/000153470126000006/psx-20251231.htm</t>
+        </is>
+      </c>
+      <c r="J98" s="6" t="inlineStr">
+        <is>
+          <t>Seminoe Montana/Wyoming 100 342 50</t>
+        </is>
+      </c>
+      <c r="K98" s="6" t="inlineStr">
+        <is>
+          <t>The EIA route layer spells it "Seminole"</t>
+        </is>
+      </c>
+      <c r="L98" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M98" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>Refined products</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>NuStar, McKee to Southlake (Dallas–Fort Worth)</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>McKee refinery (Sunray, TX) to Southlake, TX</t>
+        </is>
+      </c>
+      <c r="D99" s="9" t="n">
+        <v>26000</v>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>Official (EIA study)</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>EIA, East Coast and Gulf Coast Transportation Fuels Markets (prepared by ICF), Feb 2016, Table 30</t>
+        </is>
+      </c>
+      <c r="I99" s="10" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/analysis/transportationfuels/padd1n3/pdf/transportation_fuels_padd1n3.pdf</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>McKee, TX Southlake, TX 375 26,000</t>
+        </is>
+      </c>
+      <c r="K99" s="2" t="inlineStr"/>
+      <c r="L99" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M99" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="6" t="inlineStr">
+        <is>
+          <t>Refined products</t>
+        </is>
+      </c>
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>NuStar, McKee to El Paso</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="inlineStr">
+        <is>
+          <t>McKee refinery (Sunray, TX) to El Paso, TX</t>
+        </is>
+      </c>
+      <c r="D100" s="7" t="n">
+        <v>42000</v>
+      </c>
+      <c r="E100" s="6" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F100" s="6" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="G100" s="6" t="inlineStr">
+        <is>
+          <t>Official (EIA study)</t>
+        </is>
+      </c>
+      <c r="H100" s="6" t="inlineStr">
+        <is>
+          <t>EIA, East Coast and Gulf Coast Transportation Fuels Markets (prepared by ICF), Feb 2016, Table 30</t>
+        </is>
+      </c>
+      <c r="I100" s="8" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/analysis/transportationfuels/padd1n3/pdf/transportation_fuels_padd1n3.pdf</t>
+        </is>
+      </c>
+      <c r="J100" s="6" t="inlineStr">
+        <is>
+          <t>McKee, TX El Paso, TX 408 42,000</t>
+        </is>
+      </c>
+      <c r="K100" s="6" t="inlineStr"/>
+      <c r="L100" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M100" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>Refined products</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>NuStar, Three Rivers to San Antonio</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>Three Rivers, TX to San Antonio, TX</t>
+        </is>
+      </c>
+      <c r="D101" s="9" t="n">
+        <v>33500</v>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>Official (EIA study)</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>EIA, East Coast and Gulf Coast Transportation Fuels Markets (prepared by ICF), Feb 2016, Table 26</t>
+        </is>
+      </c>
+      <c r="I101" s="10" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/analysis/transportationfuels/padd1n3/pdf/transportation_fuels_padd1n3.pdf</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>Three Rivers, TX San Antonio, TX 85 33,500</t>
+        </is>
+      </c>
+      <c r="K101" s="2" t="inlineStr"/>
+      <c r="L101" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M101" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="6" t="inlineStr">
+        <is>
+          <t>Crude oil</t>
+        </is>
+      </c>
+      <c r="B102" s="6" t="inlineStr">
+        <is>
+          <t>Keystone Pipeline, Steele City to Patoka</t>
+        </is>
+      </c>
+      <c r="C102" s="6" t="inlineStr">
+        <is>
+          <t>Steele City, NE to Patoka, IL</t>
+        </is>
+      </c>
+      <c r="D102" s="7" t="n">
+        <v>435000</v>
+      </c>
+      <c r="E102" s="6" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F102" s="6" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="G102" s="6" t="inlineStr">
+        <is>
+          <t>Official (EIA)</t>
+        </is>
+      </c>
+      <c r="H102" s="6" t="inlineStr">
+        <is>
+          <t>EIA, Liquids pipeline projects database (ID 2)</t>
+        </is>
+      </c>
+      <c r="I102" s="8" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/petroleum/xls/EIA_LiqPipProject.xlsx</t>
+        </is>
+      </c>
+      <c r="J102" s="6" t="inlineStr">
+        <is>
+          <t>Goes from Hardisty in Alberta, Canada, down through Steele City, Nebraska, and to Patoka, Illinois. [Added capacity 435,000 b/d]</t>
+        </is>
+      </c>
+      <c r="K102" s="6" t="inlineStr"/>
+      <c r="L102" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M102" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>Crude oil</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>Keystone Pipeline, Steele City to Cushing</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>Steele City, NE to Cushing, OK</t>
+        </is>
+      </c>
+      <c r="D103" s="9" t="n">
+        <v>156000</v>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>Official (EIA)</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>EIA, Liquids pipeline projects database (ID 3)</t>
+        </is>
+      </c>
+      <c r="I103" s="10" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/petroleum/xls/EIA_LiqPipProject.xlsx</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t>Extended existing pipeline from Steele City, Nebraska, to Cushing, Oklahoma, and brought capacity of the entire system up to 591,000 b/d. [Added capacity 156,000 b/d]</t>
+        </is>
+      </c>
+      <c r="K103" s="2" t="inlineStr"/>
+      <c r="L103" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M103" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="6" t="inlineStr">
+        <is>
+          <t>Crude oil</t>
+        </is>
+      </c>
+      <c r="B104" s="6" t="inlineStr">
+        <is>
+          <t>Zydeco Pipeline (Houston to Houma)</t>
+        </is>
+      </c>
+      <c r="C104" s="6" t="inlineStr">
+        <is>
+          <t>Houston, TX via Port Neches, TX to Houma, LA</t>
+        </is>
+      </c>
+      <c r="D104" s="7" t="n">
+        <v>375000</v>
+      </c>
+      <c r="E104" s="6" t="inlineStr">
+        <is>
+          <t>Capacity (Port Neches to Houma segment)</t>
+        </is>
+      </c>
+      <c r="F104" s="6" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="G104" s="6" t="inlineStr">
+        <is>
+          <t>Official (EIA)</t>
+        </is>
+      </c>
+      <c r="H104" s="6" t="inlineStr">
+        <is>
+          <t>EIA, Liquids pipeline projects database (IDs 36 and 114)</t>
+        </is>
+      </c>
+      <c r="I104" s="8" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/petroleum/xls/EIA_LiqPipProject.xlsx</t>
+        </is>
+      </c>
+      <c r="J104" s="6" t="inlineStr">
+        <is>
+          <t>Increased capacity of Port Neches, Texas, to Houma, Louisiana, segment from 360,000 b/d to 375,000 b/d.</t>
+        </is>
+      </c>
+      <c r="K104" s="6" t="inlineStr">
+        <is>
+          <t>Houston to Port Neches segment: 250,000 b/d (ID 36)</t>
+        </is>
+      </c>
+      <c r="L104" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M104" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>Crude oil</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Permian Express 2</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>Colorado City, TX to Corsicana, TX</t>
+        </is>
+      </c>
+      <c r="D105" s="9" t="n">
+        <v>230000</v>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>Official (EIA)</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>EIA, Liquids pipeline projects database (ID 84)</t>
+        </is>
+      </c>
+      <c r="I105" s="10" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/petroleum/xls/EIA_LiqPipProject.xlsx</t>
+        </is>
+      </c>
+      <c r="J105" s="2" t="inlineStr">
+        <is>
+          <t>Garden City, Texas, to Colorado City, Texas, segment has 20-inch diameter pipeline, Colorado City to Corsicana, Texas, has 24-inch diameter pipeline. [Added capacity 230,000 b/d]</t>
+        </is>
+      </c>
+      <c r="K105" s="2" t="inlineStr"/>
+      <c r="L105" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M105" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="6" t="inlineStr">
+        <is>
+          <t>Crude oil</t>
+        </is>
+      </c>
+      <c r="B106" s="6" t="inlineStr">
+        <is>
+          <t>Marathon, Patoka to Catlettsburg</t>
+        </is>
+      </c>
+      <c r="C106" s="6" t="inlineStr">
+        <is>
+          <t>Patoka, IL via Owensboro, KY to Catlettsburg, KY</t>
+        </is>
+      </c>
+      <c r="D106" s="7" t="n">
+        <v>270000</v>
+      </c>
+      <c r="E106" s="6" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F106" s="6" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="G106" s="6" t="inlineStr">
+        <is>
+          <t>Official (EIA)</t>
+        </is>
+      </c>
+      <c r="H106" s="6" t="inlineStr">
+        <is>
+          <t>EIA, Liquids pipeline projects database (ID 22)</t>
+        </is>
+      </c>
+      <c r="I106" s="8" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/petroleum/xls/EIA_LiqPipProject.xlsx</t>
+        </is>
+      </c>
+      <c r="J106" s="6" t="inlineStr">
+        <is>
+          <t>Capacity increased from 256,000 b/d to 270,000 b/d.</t>
+        </is>
+      </c>
+      <c r="K106" s="6" t="inlineStr"/>
+      <c r="L106" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M106" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>Crude oil</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>Marathon, Patoka to Lima and Canton</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>Patoka, IL to Lima and Canton, OH</t>
+        </is>
+      </c>
+      <c r="D107" s="9" t="n">
+        <v>267000</v>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>Capacity (Patoka to Lima)</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>Official (EIA)</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>EIA, Liquids pipeline projects database (ID 111)</t>
+        </is>
+      </c>
+      <c r="I107" s="10" t="inlineStr">
+        <is>
+          <t>https://www.eia.gov/petroleum/xls/EIA_LiqPipProject.xlsx</t>
+        </is>
+      </c>
+      <c r="J107" s="2" t="inlineStr">
+        <is>
+          <t>Capacity increased from 249,000 b/d to 267,000 b/d.</t>
+        </is>
+      </c>
+      <c r="K107" s="2" t="inlineStr">
+        <is>
+          <t>EIA route continues past Lima to Canton</t>
+        </is>
+      </c>
+      <c r="L107" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M107" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="6" t="inlineStr">
+        <is>
+          <t>Crude oil</t>
+        </is>
+      </c>
+      <c r="B108" s="6" t="inlineStr">
+        <is>
+          <t>Red River Pipeline</t>
+        </is>
+      </c>
+      <c r="C108" s="6" t="inlineStr">
+        <is>
+          <t>Cushing, OK to Longview, TX</t>
+        </is>
+      </c>
+      <c r="D108" s="7" t="n">
+        <v>235000</v>
+      </c>
+      <c r="E108" s="6" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F108" s="6" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G108" s="6" t="inlineStr">
+        <is>
+          <t>Company SEC filing</t>
+        </is>
+      </c>
+      <c r="H108" s="6" t="inlineStr">
+        <is>
+          <t>Plains All American, Form 10-K for 2025</t>
+        </is>
+      </c>
+      <c r="I108" s="8" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1070423/000107042326000014/paa-20251231.htm</t>
+        </is>
+      </c>
+      <c r="J108" s="6" t="inlineStr">
+        <is>
+          <t>The Red River Pipeline is an approximately 235,000 barrel per day capacity pipeline that extends from our Cushing Terminal in Oklahoma to Longview, Texas</t>
+        </is>
+      </c>
+      <c r="K108" s="6" t="inlineStr">
+        <is>
+          <t>EIA route layer label: "CK Red River"</t>
+        </is>
+      </c>
+      <c r="L108" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M108" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>Crude oil</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>Phillips 66 Oklahoma Crude system</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>Wichita Falls, TX to Ponca City, OK</t>
+        </is>
+      </c>
+      <c r="D109" s="9" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>Company SEC filing</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>Phillips 66, Form 10-K for 2025, pipeline table</t>
+        </is>
+      </c>
+      <c r="I109" s="10" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1534701/000153470126000006/psx-20251231.htm</t>
+        </is>
+      </c>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
+          <t>Oklahoma Crude Texas/Oklahoma 100 217 100</t>
+        </is>
+      </c>
+      <c r="K109" s="2" t="inlineStr">
+        <is>
+          <t>Matched to the EIA route by operator and endpoints</t>
+        </is>
+      </c>
+      <c r="L109" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M109" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="6" t="inlineStr">
+        <is>
+          <t>Crude oil</t>
+        </is>
+      </c>
+      <c r="B110" s="6" t="inlineStr">
+        <is>
+          <t>Phillips 66 West Texas Crude system</t>
+        </is>
+      </c>
+      <c r="C110" s="6" t="inlineStr">
+        <is>
+          <t>Odessa, TX to Borger, TX</t>
+        </is>
+      </c>
+      <c r="D110" s="7" t="n">
+        <v>140000</v>
+      </c>
+      <c r="E110" s="6" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F110" s="6" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G110" s="6" t="inlineStr">
+        <is>
+          <t>Company SEC filing</t>
+        </is>
+      </c>
+      <c r="H110" s="6" t="inlineStr">
+        <is>
+          <t>Phillips 66, Form 10-K for 2025, pipeline table</t>
+        </is>
+      </c>
+      <c r="I110" s="8" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1534701/000153470126000006/psx-20251231.htm</t>
+        </is>
+      </c>
+      <c r="J110" s="6" t="inlineStr">
+        <is>
+          <t>West Texas Crude Texas 100 1,079 140</t>
+        </is>
+      </c>
+      <c r="K110" s="6" t="inlineStr">
+        <is>
+          <t>Matched to the EIA route by operator and endpoints</t>
+        </is>
+      </c>
+      <c r="L110" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M110" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>Crude oil</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>Phillips 66 California Line 200</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>San Joaquin Valley to Rodeo (San Francisco Bay), CA</t>
+        </is>
+      </c>
+      <c r="D111" s="9" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>Company SEC filing</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>Phillips 66, Form 10-K for 2025, pipeline table</t>
+        </is>
+      </c>
+      <c r="I111" s="10" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1534701/000153470126000006/psx-20251231.htm</t>
+        </is>
+      </c>
+      <c r="J111" s="2" t="inlineStr">
+        <is>
+          <t>Line 200 California 100 228 100</t>
+        </is>
+      </c>
+      <c r="K111" s="2" t="inlineStr">
+        <is>
+          <t>Matched to the EIA route by operator and endpoints</t>
+        </is>
+      </c>
+      <c r="L111" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M111" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="6" t="inlineStr">
+        <is>
+          <t>Crude oil</t>
+        </is>
+      </c>
+      <c r="B112" s="6" t="inlineStr">
+        <is>
+          <t>Trans Mountain Pipeline</t>
+        </is>
+      </c>
+      <c r="C112" s="6" t="inlineStr">
+        <is>
+          <t>Edmonton, AB to Burnaby (Vancouver), BC</t>
+        </is>
+      </c>
+      <c r="D112" s="7" t="n">
+        <v>890000</v>
+      </c>
+      <c r="E112" s="6" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="F112" s="6" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="G112" s="6" t="inlineStr">
+        <is>
+          <t>Official (Canada Energy Regulator)</t>
+        </is>
+      </c>
+      <c r="H112" s="6" t="inlineStr">
+        <is>
+          <t>Canada Energy Regulator, Market Snapshot (2025): Trans Mountain Expansion eases pipeline constraints</t>
+        </is>
+      </c>
+      <c r="I112" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cer-rec.gc.ca/en/data-analysis/energy-markets/market-snapshots/2025/market-snapshot-trans-mountain-expansion-eases-pipeline-constraints-and-increases-exports-to-overseas-markets.html</t>
+        </is>
+      </c>
+      <c r="J112" s="6" t="inlineStr">
+        <is>
+          <t>The Trans Mountain Expansion Project came online in May 2024, nearly tripling the capacity of the Trans Mountain System to a total of 890 thousand barrels per day.</t>
+        </is>
+      </c>
+      <c r="K112" s="6" t="inlineStr">
+        <is>
+          <t>Now owned by Trans Mountain Corporation (Canadian government); the EIA layer still lists Kinder Morgan. Also listed in EIA's product layer, where it is left off to avoid drawing it twice</t>
+        </is>
+      </c>
+      <c r="L112" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M112" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M96"/>
+  <autoFilter ref="A1:M112"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId2"/>
@@ -6528,6 +7508,22 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I94" r:id="rId93"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I95" r:id="rId94"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I104" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I107" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I108" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I112" r:id="rId111"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>